<commit_message>
Rebuild 2026-09-11 report with updated source exports
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B5kikMeZ9L1uCyyMsEAbgL
</commit_message>
<xml_diff>
--- a/HAL Stock HQ - Daily 2026-09-11.xlsx
+++ b/HAL Stock HQ - Daily 2026-09-11.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Daily" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RF SEASONAL" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NEW FORMAT" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Daily" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="RF SEASONAL" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="NEW FORMAT" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -1973,53 +1973,6 @@
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors/>
 </styleSheet>
-</file>
-
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <twoCellAnchor editAs="oneCell">
-    <from>
-      <col>4</col>
-      <colOff>197381</colOff>
-      <row>0</row>
-      <rowOff>7864</rowOff>
-    </from>
-    <to>
-      <col>18</col>
-      <colOff>41539</colOff>
-      <row>0</row>
-      <rowOff>590347</rowOff>
-    </to>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="3" name="Picture 2" descr="cid:image001.jpg@01D9A2D1.F406A100"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
-        <a:srcRect xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr bwMode="auto">
-        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:off x="2483381" y="7864"/>
-          <a:ext cx="4564325" cy="582483"/>
-        </a:xfrm>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:noFill/>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </twoCellAnchor>
-</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3284,7 +3237,7 @@
       <c r="AO13" s="52" t="n"/>
       <c r="AR13" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t> </t>
         </is>
       </c>
     </row>
@@ -5240,7 +5193,7 @@
       </c>
       <c r="AS39" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">   </t>
+          <t>   </t>
         </is>
       </c>
     </row>
@@ -7200,7 +7153,6 @@
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0" right="0" top="0.5" bottom="0" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" paperSize="9" scale="60"/>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>